<commit_message>
CLM: fix normative product transitions
</commit_message>
<xml_diff>
--- a/technologies/06_CLM/30 Документация/10 Диагностика/Управление_Директорами_CLM_Продукт_01_Диагностика_рабочая_книга_V1.xlsx
+++ b/technologies/06_CLM/30 Документация/10 Диагностика/Управление_Директорами_CLM_Продукт_01_Диагностика_рабочая_книга_V1.xlsx
@@ -1,185 +1,193 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
-  <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Индекс" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Первичный запрос" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Допуск" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Роли и мандаты" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Разрывы CLM" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Вердикт" sheetId="6" state="visible" r:id="rId6"/>
-  </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
-</workbook>
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:workbookPr/>
+  <x:workbookProtection/>
+  <x:bookViews>
+    <x:workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </x:bookViews>
+  <x:sheets>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Индекс" sheetId="1" state="visible" r:id="rId1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Первичный запрос" sheetId="2" state="visible" r:id="rId2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Допуск" sheetId="3" state="visible" r:id="rId3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Роли и мандаты" sheetId="4" state="visible" r:id="rId4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Разрывы CLM" sheetId="5" state="visible" r:id="rId5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Вердикт" sheetId="6" state="visible" r:id="rId6"/>
+  </x:sheets>
+  <x:definedNames/>
+  <x:calcPr calcId="124519" fullCalcOnLoad="1"/>
+</x:workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="4">
-    <font>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="0016324F"/>
-      <sz val="12"/>
-    </font>
-  </fonts>
-  <fills count="4">
-    <fill>
-      <patternFill/>
-    </fill>
-    <fill>
-      <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0016324F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF7E6"/>
-      </patternFill>
-    </fill>
-  </fills>
-  <borders count="2">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CBD5E0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CBD5E0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E0"/>
-      </bottom>
-    </border>
-  </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-  </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-  </cellXfs>
-  <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
-  </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
-</styleSheet>
+<x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="0"/>
+  <x:fonts count="4">
+    <x:font>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+      <x:color theme="1"/>
+      <x:sz val="11"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:name val="Arial"/>
+      <x:sz val="10"/>
+    </x:font>
+    <x:font>
+      <x:name val="Arial"/>
+      <x:b val="1"/>
+      <x:color rgb="00FFFFFF"/>
+      <x:sz val="10"/>
+    </x:font>
+    <x:font>
+      <x:name val="Arial"/>
+      <x:b val="1"/>
+      <x:color rgb="0016324F"/>
+      <x:sz val="12"/>
+    </x:font>
+  </x:fonts>
+  <x:fills count="5">
+    <x:fill>
+      <x:patternFill/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="0016324F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="00FFF7E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7E6"/>
+      </x:patternFill>
+    </x:fill>
+  </x:fills>
+  <x:borders count="2">
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="00CBD5E0"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="00CBD5E0"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="00CBD5E0"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="00CBD5E0"/>
+      </x:bottom>
+    </x:border>
+  </x:borders>
+  <x:cellStyleXfs count="1">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </x:cellStyleXfs>
+  <x:cellXfs count="7">
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="0" pivotButton="0"/>
+    <x:xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="0" pivotButton="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyFill="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+  </x:cellXfs>
+  <x:cellStyles count="1">
+    <x:cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </x:cellStyles>
+  <x:tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <x:colors>
+    <x:indexedColors>
+      <x:rgbColor rgb="00000000"/>
+      <x:rgbColor rgb="00FFFFFF"/>
+      <x:rgbColor rgb="00FF0000"/>
+      <x:rgbColor rgb="0000FF00"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00000000"/>
+      <x:rgbColor rgb="00FFFFFF"/>
+      <x:rgbColor rgb="00FF0000"/>
+      <x:rgbColor rgb="0000FF00"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00800000"/>
+      <x:rgbColor rgb="00008000"/>
+      <x:rgbColor rgb="00000080"/>
+      <x:rgbColor rgb="00808000"/>
+      <x:rgbColor rgb="00800080"/>
+      <x:rgbColor rgb="00008080"/>
+      <x:rgbColor rgb="00C0C0C0"/>
+      <x:rgbColor rgb="00808080"/>
+      <x:rgbColor rgb="009999FF"/>
+      <x:rgbColor rgb="00993366"/>
+      <x:rgbColor rgb="00FFFFCC"/>
+      <x:rgbColor rgb="00CCFFFF"/>
+      <x:rgbColor rgb="00660066"/>
+      <x:rgbColor rgb="00FF8080"/>
+      <x:rgbColor rgb="000066CC"/>
+      <x:rgbColor rgb="00CCCCFF"/>
+      <x:rgbColor rgb="00000080"/>
+      <x:rgbColor rgb="00FF00FF"/>
+      <x:rgbColor rgb="00FFFF00"/>
+      <x:rgbColor rgb="0000FFFF"/>
+      <x:rgbColor rgb="00800080"/>
+      <x:rgbColor rgb="00800000"/>
+      <x:rgbColor rgb="00008080"/>
+      <x:rgbColor rgb="000000FF"/>
+      <x:rgbColor rgb="0000CCFF"/>
+      <x:rgbColor rgb="00CCFFFF"/>
+      <x:rgbColor rgb="00CCFFCC"/>
+      <x:rgbColor rgb="00FFFF99"/>
+      <x:rgbColor rgb="0099CCFF"/>
+      <x:rgbColor rgb="00FF99CC"/>
+      <x:rgbColor rgb="00CC99FF"/>
+      <x:rgbColor rgb="00FFCC99"/>
+      <x:rgbColor rgb="003366FF"/>
+      <x:rgbColor rgb="0033CCCC"/>
+      <x:rgbColor rgb="0099CC00"/>
+      <x:rgbColor rgb="00FFCC00"/>
+      <x:rgbColor rgb="00FF9900"/>
+      <x:rgbColor rgb="00FF6600"/>
+      <x:rgbColor rgb="00666699"/>
+      <x:rgbColor rgb="00969696"/>
+      <x:rgbColor rgb="00003366"/>
+      <x:rgbColor rgb="00339966"/>
+      <x:rgbColor rgb="00003300"/>
+      <x:rgbColor rgb="00333300"/>
+      <x:rgbColor rgb="00993300"/>
+      <x:rgbColor rgb="00993366"/>
+      <x:rgbColor rgb="00333399"/>
+      <x:rgbColor rgb="00333333"/>
+    </x:indexedColors>
+  </x:colors>
+</x:styleSheet>
 </file>
 
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1247,129 +1255,131 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Вердикт</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Условия</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Почему</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Следующий шаг</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Кто подтверждает</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>GO / запускать</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr"/>
-      <c r="C2" s="4" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Сессия</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>GO при условиях</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr"/>
-      <c r="C3" s="4" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Сессия после условий</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Stop / остановить</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr"/>
-      <c r="C4" s="4" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Не продолжать</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="n"/>
-      <c r="B6" s="3" t="n"/>
-      <c r="C6" s="3" t="n"/>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="n"/>
-      <c r="B7" s="3" t="n"/>
-      <c r="C7" s="3" t="n"/>
-      <c r="D7" s="3" t="n"/>
-      <c r="E7" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="A2:A200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"не начато,в работе,готово,риск,Stop / остановить"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter>
-    <oddHeader>&amp;CУправление Директорами</oddHeader>
-    <oddFooter>&amp;CТехнологическая основа: CLM / C-Level Management / управление C-level-ядром.</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
-</worksheet>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+    <x:pageSetUpPr/>
+  </x:sheetPr>
+  <x:dimension ref="A1:E7"/>
+  <x:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" customWidth="1"/>
+    <x:col min="2" max="2" width="22" customWidth="1"/>
+    <x:col min="3" max="3" width="22" customWidth="1"/>
+    <x:col min="4" max="4" width="22" customWidth="1"/>
+    <x:col min="5" max="5" width="22" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Вердикт</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B1" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Условия</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C1" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Почему</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D1" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Следующий шаг</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E1" s="1" t="inlineStr">
+        <x:is>
+          <x:t>Кто подтверждает</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="2" t="inlineStr">
+        <x:is>
+          <x:t>GO / запускать</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B2" s="4" t="inlineStr"/>
+      <x:c r="C2" s="4" t="inlineStr"/>
+      <x:c r="D2" s="2" t="inlineStr">
+        <x:is>
+          <x:t>Сессия</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E2" s="4" t="inlineStr"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="2" t="inlineStr">
+        <x:is>
+          <x:t>GO при условиях</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B3" s="4" t="inlineStr"/>
+      <x:c r="C3" s="4" t="inlineStr"/>
+      <x:c r="D3" s="2" t="str">
+        <x:v>Закрыть условия → Сессия</x:v>
+      </x:c>
+      <x:c r="E3" s="4" t="inlineStr"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="2" t="str">
+        <x:v>HOLD / отложить</x:v>
+      </x:c>
+      <x:c r="B4" s="4" t="inlineStr"/>
+      <x:c r="C4" s="4" t="inlineStr"/>
+      <x:c r="D4" s="2" t="str">
+        <x:v>Вернуться в Диагностику после восстановления условий</x:v>
+      </x:c>
+      <x:c r="E4" s="4" t="inlineStr"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="6" t="str">
+        <x:v>STOP / остановить</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="n"/>
+      <x:c r="C5" s="3" t="n"/>
+      <x:c r="D5" s="6" t="str">
+        <x:v>Завершить</x:v>
+      </x:c>
+      <x:c r="E5" s="3" t="n"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="6" t="str">
+        <x:v>NO FIT / не подходит</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="n"/>
+      <x:c r="C6" s="3" t="n"/>
+      <x:c r="D6" s="6" t="str">
+        <x:v>Завершить</x:v>
+      </x:c>
+      <x:c r="E6" s="3" t="n"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="3" t="n"/>
+      <x:c r="B7" s="3" t="n"/>
+      <x:c r="C7" s="3" t="n"/>
+      <x:c r="D7" s="3" t="n"/>
+      <x:c r="E7" s="3" t="n"/>
+    </x:row>
+  </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" allowBlank="1" showDropDown="0" showInputMessage="0" showErrorMessage="0" sqref="A2:A200">
+      <x:formula1>"не начато,в работе,готово,риск,Stop / остановить"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <x:headerFooter>
+    <x:oddHeader>&amp;CУправление Директорами</x:oddHeader>
+    <x:oddFooter>&amp;CТехнологическая основа: CLM / C-Level Management / управление C-level-ядром.</x:oddFooter>
+    <x:evenHeader/>
+    <x:evenFooter/>
+    <x:firstHeader/>
+    <x:firstFooter/>
+  </x:headerFooter>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</x:worksheet>
 </file>
</xml_diff>